<commit_message>
Update Louis Htoo plan from handwritten notes — 17:00 start, 19-item flow
Completely revised party plan based on handwritten schedule:
- Start time moved to 17:00 (party ends 20:00)
- Prep from 15:20: uketsuke 15:30, group photo 2F, chapel photoshoot 16:10-16:30
- Full ceremony within reception: slideshow → groom/bride entrance → virgin road
  → 15min ceremony → kanpai (Mg Mg Phyo) → cake (first bite + first kiss + rings)
  → couple exit (flash phone lights) → chuza entertainment (game paper + glow stick
  + AI movie) → re-entrance (laser show + stairs + love speech) → MC quiz (10Q)
  → table round → bride letter → groom speech → flower shower → bouquet toss
  (from stairs) → group photo → depart (1 door) → lobby petit gift

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="102">
   <si>
     <t>Hotel Bell Classic_WEDDING PARTY PLAN</t>
   </si>
@@ -79,184 +79,244 @@
     <t>BGM</t>
   </si>
   <si>
-    <t>16:00</t>
-  </si>
-  <si>
-    <t>会場準備</t>
+    <t>15:20</t>
+  </si>
+  <si>
+    <t>ゲスト受付</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>[Staff]</t>
+    <t>[Receptionist] 15:30 First meet — Video &amp; Photo team on standby</t>
+  </si>
+  <si>
+    <t>15:50</t>
+  </si>
+  <si>
+    <t>集合写真（2F）</t>
+  </si>
+  <si>
+    <t>[Photographer] 15:45 — 2F group photo with guests</t>
+  </si>
+  <si>
+    <t>16:15</t>
+  </si>
+  <si>
+    <t>チャペル撮影</t>
+  </si>
+  <si>
+    <t>[Photographer] 16:10~16:30 chapel photoshoot — then couple rests</t>
+  </si>
+  <si>
+    <t>16:35</t>
+  </si>
+  <si>
+    <t>MC準備・BGM確認</t>
+  </si>
+  <si>
+    <t>[MC] 16:00 MC spare check / 16:30 MC confirm BGM</t>
+  </si>
+  <si>
+    <t>16:50</t>
+  </si>
+  <si>
+    <t>入場待機</t>
+  </si>
+  <si>
+    <t>[Couple]</t>
   </si>
   <si>
     <t>17:00</t>
   </si>
   <si>
-    <t>ゲスト受付</t>
-  </si>
-  <si>
-    <t>[Receptionist]</t>
-  </si>
-  <si>
-    <t>17:30</t>
-  </si>
-  <si>
-    <t>お二人写真撮影（記念orスナップ）</t>
+    <t>スライドショー上映</t>
+  </si>
+  <si>
+    <t>[Tech] ~5 min slideshow before entrance begins</t>
+  </si>
+  <si>
+    <t>① Slideshow BGM</t>
+  </si>
+  <si>
+    <t>17:05</t>
+  </si>
+  <si>
+    <t>新郎入場（友人と共に） 🎭</t>
+  </si>
+  <si>
+    <t>[Groom] Groom enters with friends → waits at middle of 1F</t>
+  </si>
+  <si>
+    <t>② Groom Entrance BGM</t>
+  </si>
+  <si>
+    <t>17:10</t>
+  </si>
+  <si>
+    <t>新婦入場（父と共に）・バージンロードへ 🎭</t>
+  </si>
+  <si>
+    <t>[Bride] Bride enters with father → father handover to groom</t>
+  </si>
+  <si>
+    <t>③ Bride Entrance BGM</t>
+  </si>
+  <si>
+    <t>17:15</t>
+  </si>
+  <si>
+    <t>お二人でバージンロード 🎭</t>
+  </si>
+  <si>
+    <t>④ Virgin Road BGM</t>
+  </si>
+  <si>
+    <t>17:20</t>
+  </si>
+  <si>
+    <t>挙式 🎤 🎭</t>
+  </si>
+  <si>
+    <t>[MC] 15 min — Louis (groom) active role. Mg Mg Phyo officiating (3 people on stage)</t>
+  </si>
+  <si>
+    <t>17:35</t>
+  </si>
+  <si>
+    <t>乾杯・ウェルカムスピーチ 🎤 🎭</t>
+  </si>
+  <si>
+    <t>[Guest (Friend)] Friend (Mg Mg Phyo) gives welcome speech → Kanpai</t>
+  </si>
+  <si>
+    <t>17:40</t>
+  </si>
+  <si>
+    <t>ケーキ入刀・ファーストバイト・ファーストキス・指輪お披露目 🎭</t>
+  </si>
+  <si>
+    <t>[Couple] Sequence: Cake cutting → First bite (groom→bride) → First kiss → Ring reveal</t>
+  </si>
+  <si>
+    <t>⑤ Cake BGM</t>
+  </si>
+  <si>
+    <t>17:50</t>
+  </si>
+  <si>
+    <t>新郎新婦中座（フラッシュライト演出） 🎭</t>
+  </si>
+  <si>
+    <t>[Couple] Guests hold up phone flashlights to send off couple for costume change</t>
+  </si>
+  <si>
+    <t>17:55</t>
+  </si>
+  <si>
+    <t>中座余興 — ゲーム用紙・グロースティック配布・AI映像上映</t>
+  </si>
+  <si>
+    <t>[MC / Tech] Distribute game paper + glow sticks to all guests. AI movie/profile video plays during costume change.</t>
+  </si>
+  <si>
+    <t>18:10</t>
+  </si>
+  <si>
+    <t>再入場 — レーザーショー・階段・ラブスピーチ（グロースティック） 🎭</t>
+  </si>
+  <si>
+    <t>[Couple] Laser show → couple descends from stairs → Love speech with glow sticks lit by guests</t>
+  </si>
+  <si>
+    <t>⑥ Re-entrance BGM</t>
+  </si>
+  <si>
+    <t>18:20</t>
+  </si>
+  <si>
+    <t>ゲーム — MCクイズ（10問） 🎤 🎭</t>
+  </si>
+  <si>
+    <t>[MC] 10 questions about the couple. Guest with &gt; 5 correct answers wins a gift. (Louis provides gifts)</t>
+  </si>
+  <si>
+    <t>18:35</t>
+  </si>
+  <si>
+    <t>カミングフォト（テーブルラウンド）</t>
+  </si>
+  <si>
+    <t>[Couple / Photo] Couple visits each table for photos with guests</t>
+  </si>
+  <si>
+    <t>18:50</t>
+  </si>
+  <si>
+    <t>新婦から家族への手紙 🎤 🎭</t>
+  </si>
+  <si>
+    <t>[Bride]</t>
+  </si>
+  <si>
+    <t>18:55</t>
+  </si>
+  <si>
+    <t>新郎謝辞 🎤 🎭</t>
+  </si>
+  <si>
+    <t>[Groom]</t>
+  </si>
+  <si>
+    <t>19:00</t>
+  </si>
+  <si>
+    <t>フラワーシャワー 🎭</t>
+  </si>
+  <si>
+    <t>[Guests] Flower shower — highlighted as key moment</t>
+  </si>
+  <si>
+    <t>⑦ Flower Shower BGM</t>
+  </si>
+  <si>
+    <t>19:05</t>
+  </si>
+  <si>
+    <t>ブーケトス（階段より） 🎭</t>
+  </si>
+  <si>
+    <t>[Bride] Bride throws bouquet from top of stairs down to guests at ground level</t>
+  </si>
+  <si>
+    <t>19:15</t>
+  </si>
+  <si>
+    <t>全員集合写真</t>
   </si>
   <si>
     <t>[Photographer]</t>
   </si>
   <si>
-    <t>17:50</t>
-  </si>
-  <si>
-    <t>入場待機</t>
-  </si>
-  <si>
-    <t>[Couple]</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>披露宴スタート 🎤</t>
-  </si>
-  <si>
-    <t>[MC]</t>
-  </si>
-  <si>
-    <t>18:05</t>
-  </si>
-  <si>
-    <t>新郎新婦入場 🎭</t>
-  </si>
-  <si>
-    <t>① Entrance BGM</t>
-  </si>
-  <si>
-    <t>18:10</t>
-  </si>
-  <si>
-    <t>ウェルカムスピーチ・乾杯 🎤 🎭</t>
-  </si>
-  <si>
-    <t>18:15</t>
-  </si>
-  <si>
-    <t>ケーキ入刀 🎭</t>
-  </si>
-  <si>
-    <t>② Cake Cutting BGM</t>
-  </si>
-  <si>
-    <t>18:20</t>
-  </si>
-  <si>
-    <t>ファーストバイト 🎭</t>
-  </si>
-  <si>
-    <t>18:25</t>
-  </si>
-  <si>
-    <t>食事START!</t>
-  </si>
-  <si>
-    <t>[Venue]</t>
-  </si>
-  <si>
-    <t>18:30</t>
-  </si>
-  <si>
-    <t>新郎新婦プロフィール紹介 🎤 🎭</t>
-  </si>
-  <si>
-    <t>18:40</t>
-  </si>
-  <si>
-    <t>食事・歓談</t>
-  </si>
-  <si>
-    <t>19:10</t>
-  </si>
-  <si>
-    <t>スピーチ① 🎤 🎭</t>
-  </si>
-  <si>
-    <t>[Guest]</t>
-  </si>
-  <si>
-    <t>19:15</t>
-  </si>
-  <si>
-    <t>スピーチ② 🎤 🎭</t>
-  </si>
-  <si>
-    <t>19:20</t>
-  </si>
-  <si>
-    <t>映像上映・余興 🎭</t>
-  </si>
-  <si>
-    <t>[Tech]</t>
-  </si>
-  <si>
     <t>19:25</t>
   </si>
   <si>
-    <t>余興・ゲーム 🎤 🎭</t>
-  </si>
-  <si>
-    <t>19:40</t>
-  </si>
-  <si>
-    <t>新婦中座</t>
-  </si>
-  <si>
-    <t>[Bride]</t>
-  </si>
-  <si>
-    <t>19:55</t>
-  </si>
-  <si>
-    <t>プロフィールＶＴＲ上映 🎭</t>
-  </si>
-  <si>
-    <t>20:00</t>
-  </si>
-  <si>
-    <t>再入場 🎭</t>
-  </si>
-  <si>
-    <t>③ Re-entry BGM</t>
-  </si>
-  <si>
-    <t>20:05</t>
-  </si>
-  <si>
-    <t>カミングフォト</t>
-  </si>
-  <si>
-    <t>[Couple/Photo]</t>
-  </si>
-  <si>
-    <t>20:20</t>
-  </si>
-  <si>
-    <t>ブーケトス・集合写真</t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>謝辞・新郎新婦退場 🎤 🎭</t>
-  </si>
-  <si>
-    <t>20:35</t>
-  </si>
-  <si>
-    <t>送賓 (プチギフト)</t>
+    <t>新郎新婦ご退場（お二人一緒に・1ドア） 🎭</t>
+  </si>
+  <si>
+    <t>[Couple] Both exit together through 1 door</t>
+  </si>
+  <si>
+    <t>⑧ Departure BGM</t>
+  </si>
+  <si>
+    <t>19:30</t>
+  </si>
+  <si>
+    <t>ロビー送賓・プチギフト</t>
+  </si>
+  <si>
+    <t>[Couple] Couple stands at lobby entrance, gives petit gift to each departing guest</t>
   </si>
 </sst>
 </file>
@@ -869,7 +929,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="8" style="1" customWidth="1"/>
@@ -1094,7 +1154,7 @@
         <v>35</v>
       </c>
       <c r="B13" s="21"/>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="22" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="23" t="s">
@@ -1122,91 +1182,91 @@
         <v>24</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I14" s="25"/>
     </row>
     <row r="15" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="26" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D15" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="24"/>
       <c r="H15" s="25" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="I15" s="25"/>
     </row>
     <row r="16" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="26" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D16" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="F16" s="24"/>
       <c r="G16" s="24"/>
       <c r="H16" s="25" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="I16" s="25"/>
     </row>
     <row r="17" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="26" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D17" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F17" s="24"/>
       <c r="G17" s="24"/>
       <c r="H17" s="25" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="I17" s="25"/>
     </row>
     <row r="18" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="26" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D18" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F18" s="24"/>
       <c r="G18" s="24"/>
@@ -1217,17 +1277,17 @@
     </row>
     <row r="19" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B19" s="21"/>
       <c r="C19" s="26" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D19" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
@@ -1238,38 +1298,38 @@
     </row>
     <row r="20" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B20" s="21"/>
       <c r="C20" s="26" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D20" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="F20" s="24"/>
       <c r="G20" s="24"/>
       <c r="H20" s="25" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="I20" s="25"/>
     </row>
     <row r="21" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B21" s="21"/>
       <c r="C21" s="26" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D21" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
@@ -1280,17 +1340,17 @@
     </row>
     <row r="22" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="26" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D22" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="F22" s="24"/>
       <c r="G22" s="24"/>
@@ -1301,38 +1361,38 @@
     </row>
     <row r="23" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B23" s="21"/>
       <c r="C23" s="26" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="D23" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
       <c r="H23" s="25" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="I23" s="25"/>
     </row>
     <row r="24" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="26" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D24" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
@@ -1343,17 +1403,17 @@
     </row>
     <row r="25" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="B25" s="21"/>
       <c r="C25" s="26" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D25" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="F25" s="24"/>
       <c r="G25" s="24"/>
@@ -1364,17 +1424,17 @@
     </row>
     <row r="26" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B26" s="21"/>
       <c r="C26" s="26" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D26" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="F26" s="24"/>
       <c r="G26" s="24"/>
@@ -1385,59 +1445,59 @@
     </row>
     <row r="27" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B27" s="21"/>
       <c r="C27" s="26" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D27" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="F27" s="24"/>
       <c r="G27" s="24"/>
       <c r="H27" s="25" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="I27" s="25"/>
     </row>
     <row r="28" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="26" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="D28" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
       <c r="H28" s="25" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="I28" s="25"/>
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="26" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="D29" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
@@ -1448,17 +1508,17 @@
     </row>
     <row r="30" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="B30" s="21"/>
       <c r="C30" s="26" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="D30" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E30" s="24" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="F30" s="24"/>
       <c r="G30" s="24"/>
@@ -1468,28 +1528,49 @@
       <c r="I30" s="25"/>
     </row>
     <row r="31" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E31" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="I31" s="30"/>
+      <c r="A31" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="21"/>
+      <c r="C31" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="I31" s="25"/>
+    </row>
+    <row r="32" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="27"/>
+      <c r="C32" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E32" s="29" t="s">
+        <v>101</v>
+      </c>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="I32" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="87">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:D4"/>
     <mergeCell ref="F2:G2"/>
@@ -1574,6 +1655,9 @@
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="H31:I31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="H32:I32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Use language-aware name resolution for Excel export
Previously Excel always used nameJa, so edits made in English or Burmese mode
were silently ignored. Now the export mirrors the UI: uses nameEn when the plan
language is 'en', nameMy for 'my', nameJa for 'ja' — what you see is what you get.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -82,7 +82,7 @@
     <t>15:20</t>
   </si>
   <si>
-    <t>ゲスト受付</t>
+    <t>Guest Reception</t>
   </si>
   <si>
     <t/>
@@ -94,7 +94,7 @@
     <t>15:50</t>
   </si>
   <si>
-    <t>集合写真（2F）</t>
+    <t>Group Photo 2F</t>
   </si>
   <si>
     <t>[Photographer] 15:45 — 2F group photo with guests</t>
@@ -103,7 +103,7 @@
     <t>16:15</t>
   </si>
   <si>
-    <t>チャペル撮影</t>
+    <t>Chapel Photoshoot</t>
   </si>
   <si>
     <t>[Photographer] 16:10~16:30 chapel photoshoot — then couple rests</t>
@@ -112,7 +112,7 @@
     <t>16:35</t>
   </si>
   <si>
-    <t>MC準備・BGM確認</t>
+    <t>MC Preparation &amp; BGM Confirm</t>
   </si>
   <si>
     <t>[MC] 16:00 MC spare check / 16:30 MC confirm BGM</t>
@@ -121,7 +121,7 @@
     <t>16:50</t>
   </si>
   <si>
-    <t>入場待機</t>
+    <t>Waiting for Entrance</t>
   </si>
   <si>
     <t>[Couple]</t>
@@ -130,7 +130,7 @@
     <t>17:00</t>
   </si>
   <si>
-    <t>スライドショー上映</t>
+    <t>Slideshow</t>
   </si>
   <si>
     <t>[Tech] ~5 min slideshow before entrance begins</t>
@@ -142,7 +142,7 @@
     <t>17:05</t>
   </si>
   <si>
-    <t>新郎入場（友人と共に） 🎭</t>
+    <t>Groom Entrance with Friends 🎭</t>
   </si>
   <si>
     <t>[Groom] Groom enters with friends → waits at middle of 1F</t>
@@ -154,7 +154,7 @@
     <t>17:10</t>
   </si>
   <si>
-    <t>新婦入場（父と共に）・バージンロードへ 🎭</t>
+    <t>Bride Entrance with Father — Handover 🎭</t>
   </si>
   <si>
     <t>[Bride] Bride enters with father → father handover to groom</t>
@@ -166,7 +166,7 @@
     <t>17:15</t>
   </si>
   <si>
-    <t>お二人でバージンロード 🎭</t>
+    <t>Together — Virgin Road 🎭</t>
   </si>
   <si>
     <t>④ Virgin Road BGM</t>
@@ -175,7 +175,7 @@
     <t>17:20</t>
   </si>
   <si>
-    <t>挙式 🎤 🎭</t>
+    <t>Ceremony 🎤 🎭</t>
   </si>
   <si>
     <t>[MC] 15 min — Louis (groom) active role. Mg Mg Phyo officiating (3 people on stage)</t>
@@ -184,7 +184,7 @@
     <t>17:35</t>
   </si>
   <si>
-    <t>乾杯・ウェルカムスピーチ 🎤 🎭</t>
+    <t>Kanpai — Welcome Toast 🎤 🎭</t>
   </si>
   <si>
     <t>[Guest (Friend)] Friend (Mg Mg Phyo) gives welcome speech → Kanpai</t>
@@ -193,7 +193,7 @@
     <t>17:40</t>
   </si>
   <si>
-    <t>ケーキ入刀・ファーストバイト・ファーストキス・指輪お披露目 🎭</t>
+    <t>Cake Cutting — First Bite, First Kiss &amp; Rings 🎭</t>
   </si>
   <si>
     <t>[Couple] Sequence: Cake cutting → First bite (groom→bride) → First kiss → Ring reveal</t>
@@ -205,7 +205,7 @@
     <t>17:50</t>
   </si>
   <si>
-    <t>新郎新婦中座（フラッシュライト演出） 🎭</t>
+    <t>Couple Exit — Flash Phone Lights 🎭</t>
   </si>
   <si>
     <t>[Couple] Guests hold up phone flashlights to send off couple for costume change</t>
@@ -214,7 +214,7 @@
     <t>17:55</t>
   </si>
   <si>
-    <t>中座余興 — ゲーム用紙・グロースティック配布・AI映像上映</t>
+    <t>Chuza Entertainment — Game Paper, Glow Sticks &amp; AI Movie</t>
   </si>
   <si>
     <t>[MC / Tech] Distribute game paper + glow sticks to all guests. AI movie/profile video plays during costume change.</t>
@@ -223,7 +223,7 @@
     <t>18:10</t>
   </si>
   <si>
-    <t>再入場 — レーザーショー・階段・ラブスピーチ（グロースティック） 🎭</t>
+    <t>Re-entrance — Laser Show, Stairs &amp; Love Speech 🎭</t>
   </si>
   <si>
     <t>[Couple] Laser show → couple descends from stairs → Love speech with glow sticks lit by guests</t>
@@ -235,7 +235,7 @@
     <t>18:20</t>
   </si>
   <si>
-    <t>ゲーム — MCクイズ（10問） 🎤 🎭</t>
+    <t>Game — MC Quiz 🎤 🎭</t>
   </si>
   <si>
     <t>[MC] 10 questions about the couple. Guest with &gt; 5 correct answers wins a gift. (Louis provides gifts)</t>
@@ -244,7 +244,7 @@
     <t>18:35</t>
   </si>
   <si>
-    <t>カミングフォト（テーブルラウンド）</t>
+    <t>Round Table Photo</t>
   </si>
   <si>
     <t>[Couple / Photo] Couple visits each table for photos with guests</t>
@@ -253,7 +253,7 @@
     <t>18:50</t>
   </si>
   <si>
-    <t>新婦から家族への手紙 🎤 🎭</t>
+    <t>Letter to Family — Bride 🎤 🎭</t>
   </si>
   <si>
     <t>[Bride]</t>
@@ -262,7 +262,7 @@
     <t>18:55</t>
   </si>
   <si>
-    <t>新郎謝辞 🎤 🎭</t>
+    <t>Thank You Message — Groom 🎤 🎭</t>
   </si>
   <si>
     <t>[Groom]</t>
@@ -271,7 +271,7 @@
     <t>19:00</t>
   </si>
   <si>
-    <t>フラワーシャワー 🎭</t>
+    <t>Flower Shower 🎭</t>
   </si>
   <si>
     <t>[Guests] Flower shower — highlighted as key moment</t>
@@ -283,7 +283,7 @@
     <t>19:05</t>
   </si>
   <si>
-    <t>ブーケトス（階段より） 🎭</t>
+    <t>Bouquet Toss from Stairs 🎭</t>
   </si>
   <si>
     <t>[Bride] Bride throws bouquet from top of stairs down to guests at ground level</t>
@@ -292,7 +292,7 @@
     <t>19:15</t>
   </si>
   <si>
-    <t>全員集合写真</t>
+    <t>Group Photo</t>
   </si>
   <si>
     <t>[Photographer]</t>
@@ -301,7 +301,7 @@
     <t>19:25</t>
   </si>
   <si>
-    <t>新郎新婦ご退場（お二人一緒に・1ドア） 🎭</t>
+    <t>Depart — Both Together 🎭</t>
   </si>
   <si>
     <t>[Couple] Both exit together through 1 door</t>
@@ -313,7 +313,7 @@
     <t>19:30</t>
   </si>
   <si>
-    <t>ロビー送賓・プチギフト</t>
+    <t>Lobby — Petit Gift Farewell</t>
   </si>
   <si>
     <t>[Couple] Couple stands at lobby entrance, gives petit gift to each departing guest</t>

</xml_diff>

<commit_message>
Update Louis Htoo plan with venue sheet notes
- Bride name filled in: Ei Phyu Win (was TBD)
- Groom official name: Tint Htoo Aung (nickname: Louis)
- Added metadata: endTime 19:30, extras (dessert buffet, table photos, after-party, flower bring-in, handmade showcase, parking, groom costume note)
- Added new activity lh-10b: Guest Speeches — Father & Friends (1-2 groups, 5 min each) after re-entrance
- Updated coordinationNotes: opening BGM Type-C, cake sequence corrected (cutting→bite→ring reveal→kiss), groom 2nd outfit T-shirt+coat, re-entrance from 2F Gallery with BGM Sweet Heart, table layout details, bride letter with BGM, farewell photo note

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
   <si>
     <t>Hotel Bell Classic_WEDDING PARTY PLAN</t>
   </si>
@@ -43,10 +43,10 @@
     <t>90  名様</t>
   </si>
   <si>
-    <t>新郎   Louis Htoo   様</t>
-  </si>
-  <si>
-    <t>新婦   TBD   様</t>
+    <t>新郎   Tint Htoo Aung   様</t>
+  </si>
+  <si>
+    <t>新婦   Ei Phyu Win   様</t>
   </si>
   <si>
     <t>VTR撮影</t>
@@ -88,7 +88,7 @@
     <t/>
   </si>
   <si>
-    <t>[Receptionist] 15:30 First meet — Video &amp; Photo team on standby</t>
+    <t>[Receptionist] 15:30 First meet — Video &amp; Photo team on standby. Venue setup: banner posters, tent cards, small tables, DMC QR code cards at each seat.</t>
   </si>
   <si>
     <t>15:50</t>
@@ -115,7 +115,7 @@
     <t>MC Preparation &amp; BGM Confirm</t>
   </si>
   <si>
-    <t>[MC] 16:00 MC spare check / 16:30 MC confirm BGM</t>
+    <t>[MC] 16:00 MC spare check / 16:30 MC confirm BGM. Confirm Type-C BGM for opening slideshow &amp; entrance.</t>
   </si>
   <si>
     <t>16:50</t>
@@ -133,10 +133,10 @@
     <t>Slideshow</t>
   </si>
   <si>
-    <t>[Tech] ~5 min slideshow before entrance begins</t>
-  </si>
-  <si>
-    <t>① Slideshow BGM</t>
+    <t>[Tech] BGM: Type-C. Slideshow of couple's lifestyle photos &amp; highlight video — plays before entrance begins.</t>
+  </si>
+  <si>
+    <t>① Type-C</t>
   </si>
   <si>
     <t>17:05</t>
@@ -145,10 +145,10 @@
     <t>Groom Entrance with Friends 🎭</t>
   </si>
   <si>
-    <t>[Groom] Groom enters with friends → waits at middle of 1F</t>
-  </si>
-  <si>
-    <t>② Groom Entrance BGM</t>
+    <t>[Groom] BGM: Type-C entrance. Groom enters with friends one by one → waits at centre of floor.</t>
+  </si>
+  <si>
+    <t>② Groom Entrance BGM (Type-C)</t>
   </si>
   <si>
     <t>17:10</t>
@@ -178,7 +178,7 @@
     <t>Ceremony 🎤 🎭</t>
   </si>
   <si>
-    <t>[MC] 15 min — Louis (groom) active role. Mg Mg Phyo officiating (3 people on stage)</t>
+    <t>[MC] 15 min. Tint Htoo Aung (groom) has active role. Mg Mg Phyo officiating — 3 people on stage.</t>
   </si>
   <si>
     <t>17:35</t>
@@ -187,7 +187,7 @@
     <t>Kanpai — Welcome Toast 🎤 🎭</t>
   </si>
   <si>
-    <t>[Guest (Friend)] Friend (Mg Mg Phyo) gives welcome speech → Kanpai</t>
+    <t>[Guest (Friend)] Friend (Mg Mg Phyo) gives welcome speech → Kanpai toast.</t>
   </si>
   <si>
     <t>17:40</t>
@@ -196,7 +196,7 @@
     <t>Cake Cutting — First Bite, First Kiss &amp; Rings 🎭</t>
   </si>
   <si>
-    <t>[Couple] Sequence: Cake cutting → First bite (groom→bride) → First kiss → Ring reveal</t>
+    <t>[Couple] Sequence (venue confirmed): Cake cutting → First bite (groom feeds bride) → Ring reveal to guests → First kiss.</t>
   </si>
   <si>
     <t>⑤ Cake BGM</t>
@@ -208,7 +208,7 @@
     <t>Couple Exit — Flash Phone Lights 🎭</t>
   </si>
   <si>
-    <t>[Couple] Guests hold up phone flashlights to send off couple for costume change</t>
+    <t>[Couple] Guests hold up phone flashlights to send off couple for costume change. Groom's 2nd outfit: T-shirt + coat.</t>
   </si>
   <si>
     <t>17:55</t>
@@ -217,7 +217,7 @@
     <t>Chuza Entertainment — Game Paper, Glow Sticks &amp; AI Movie</t>
   </si>
   <si>
-    <t>[MC / Tech] Distribute game paper + glow sticks to all guests. AI movie/profile video plays during costume change.</t>
+    <t>[MC / Tech] Distribute game quiz paper + glow sticks to ALL guests. AI/profile video plays simultaneously. Photographer takes table photos during this time.</t>
   </si>
   <si>
     <t>18:10</t>
@@ -226,40 +226,49 @@
     <t>Re-entrance — Laser Show, Stairs &amp; Love Speech 🎭</t>
   </si>
   <si>
-    <t>[Couple] Laser show → couple descends from stairs → Love speech with glow sticks lit by guests</t>
-  </si>
-  <si>
-    <t>⑥ Re-entrance BGM</t>
+    <t>[Couple] Laser show → couple descends from 2F Gallery stairs → Love speech (guests hold lit glow sticks). BGM: Sweet Heart.</t>
+  </si>
+  <si>
+    <t>⑥ Sweet Heart</t>
   </si>
   <si>
     <t>18:20</t>
   </si>
   <si>
+    <t>Guest Speeches — Father &amp; Friends 🎤 🎭</t>
+  </si>
+  <si>
+    <t>[Guest (Father / Friend)] 1–2 groups (father's side + friend's side). Each group within 5 min. MC to introduce each speaker. Couple stands at front of stage.</t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
     <t>Game — MC Quiz 🎤 🎭</t>
   </si>
   <si>
-    <t>[MC] 10 questions about the couple. Guest with &gt; 5 correct answers wins a gift. (Louis provides gifts)</t>
-  </si>
-  <si>
-    <t>18:35</t>
+    <t>[MC] 10 questions about the couple (use the game paper distributed during 中座). Guests with 5+ correct answers win a prize — couple provides prizes. Confirm rehearsal &amp; sound check with MC.</t>
+  </si>
+  <si>
+    <t>18:45</t>
   </si>
   <si>
     <t>Round Table Photo</t>
   </si>
   <si>
-    <t>[Couple / Photo] Couple visits each table for photos with guests</t>
-  </si>
-  <si>
-    <t>18:50</t>
+    <t>[Couple / Photo] Couple visits each table for photos. Table layout: approx. 10 round tables × 30 guests / 9 round tables × 36 guests. Photographer covers all tables.</t>
+  </si>
+  <si>
+    <t>19:00</t>
   </si>
   <si>
     <t>Letter to Family — Bride 🎤 🎭</t>
   </si>
   <si>
-    <t>[Bride]</t>
-  </si>
-  <si>
-    <t>18:55</t>
+    <t>[Bride] Bride reads letter to family with soft backing BGM. Tech: cue music at the start. Tissues ready.</t>
+  </si>
+  <si>
+    <t>19:05</t>
   </si>
   <si>
     <t>Thank You Message — Groom 🎤 🎭</t>
@@ -268,55 +277,55 @@
     <t>[Groom]</t>
   </si>
   <si>
-    <t>19:00</t>
+    <t>19:10</t>
   </si>
   <si>
     <t>Flower Shower 🎭</t>
   </si>
   <si>
-    <t>[Guests] Flower shower — highlighted as key moment</t>
+    <t>[Guests] Key highlight moment. Couple walks through flower shower from guests.</t>
   </si>
   <si>
     <t>⑦ Flower Shower BGM</t>
   </si>
   <si>
-    <t>19:05</t>
+    <t>19:15</t>
   </si>
   <si>
     <t>Bouquet Toss from Stairs 🎭</t>
   </si>
   <si>
-    <t>[Bride] Bride throws bouquet from top of stairs down to guests at ground level</t>
-  </si>
-  <si>
-    <t>19:15</t>
+    <t>[Bride] Bride throws bouquet from top of 2F Gallery stairs down to guests at ground floor.</t>
+  </si>
+  <si>
+    <t>19:25</t>
   </si>
   <si>
     <t>Group Photo</t>
   </si>
   <si>
-    <t>[Photographer]</t>
-  </si>
-  <si>
-    <t>19:25</t>
+    <t>[Photographer] All guests + couple + family. Photographer coordinates positioning.</t>
+  </si>
+  <si>
+    <t>19:35</t>
   </si>
   <si>
     <t>Depart — Both Together 🎭</t>
   </si>
   <si>
-    <t>[Couple] Both exit together through 1 door</t>
+    <t>[Couple] Both exit together through 1 door. Guests line both sides and applaud/wave.</t>
   </si>
   <si>
     <t>⑧ Departure BGM</t>
   </si>
   <si>
-    <t>19:30</t>
+    <t>19:40</t>
   </si>
   <si>
     <t>Lobby — Petit Gift Farewell</t>
   </si>
   <si>
-    <t>[Couple] Couple stands at lobby entrance, gives petit gift to each departing guest</t>
+    <t>[Couple] Couple stands at lobby entrance, gives petit gift to each departing guest. Photographer captures farewell moments. Party closes at 19:30.</t>
   </si>
 </sst>
 </file>
@@ -929,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="8" style="1" customWidth="1"/>
@@ -1481,28 +1490,28 @@
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
       <c r="H28" s="25" t="s">
-        <v>88</v>
+        <v>24</v>
       </c>
       <c r="I28" s="25"/>
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" s="24" t="s">
         <v>90</v>
-      </c>
-      <c r="D29" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E29" s="24" t="s">
-        <v>91</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
       <c r="H29" s="25" t="s">
-        <v>24</v>
+        <v>91</v>
       </c>
       <c r="I29" s="25"/>
     </row>
@@ -1544,33 +1553,54 @@
       <c r="F31" s="24"/>
       <c r="G31" s="24"/>
       <c r="H31" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="I31" s="25"/>
+    </row>
+    <row r="32" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="I31" s="25"/>
-    </row>
-    <row r="32" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="27" t="s">
+      <c r="B32" s="21"/>
+      <c r="C32" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="28" t="s">
+      <c r="D32" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E32" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="D32" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E32" s="29" t="s">
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="I32" s="30"/>
+      <c r="I32" s="25"/>
+    </row>
+    <row r="33" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="27"/>
+      <c r="C33" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E33" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="I33" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="87">
+  <mergeCells count="90">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:D4"/>
     <mergeCell ref="F2:G2"/>
@@ -1658,6 +1688,9 @@
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="E32:G32"/>
     <mergeCell ref="H32:I32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="H33:I33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Fix Excel column distribution and add language-aware 内容 column
- Added coordinationNotesJa/My fields to TimelineActivity, Activity types
- Excel 内容 column now uses language-aware notes: coordinationNotesJa when plan
  is set to Japanese, coordinationNotesMy for Burmese, English as fallback
- Removed 'responsible' from 内容 column — it doesn't belong there
- 場所 column now populated: added location to all Louis Htoo plan activities
- UI: location field is now editable inline (MapPin → click to edit)
- UI: coordinationNotes now visible and editable in the timeline — language-aware
  (editing in JA mode updates coordinationNotesJa, EN mode updates coordinationNotes)
- Added coordinationNotesJa (Japanese) to all Louis Htoo plan activities
- Regenerated Excel with correct column distribution

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="103">
   <si>
     <t>Hotel Bell Classic_WEDDING PARTY PLAN</t>
   </si>
@@ -88,7 +88,7 @@
     <t/>
   </si>
   <si>
-    <t>[Receptionist] 15:30 First meet — Video &amp; Photo team on standby. Venue setup: banner posters, tent cards, small tables, DMC QR code cards at each seat.</t>
+    <t>15:30 First meet — Video &amp; Photo team on standby. Venue setup: banner posters, tent cards, small tables, DMC QR code cards at each seat.</t>
   </si>
   <si>
     <t>15:50</t>
@@ -97,7 +97,7 @@
     <t>Group Photo 2F</t>
   </si>
   <si>
-    <t>[Photographer] 15:45 — 2F group photo with guests</t>
+    <t>15:45 — 2F group photo with guests</t>
   </si>
   <si>
     <t>16:15</t>
@@ -106,7 +106,7 @@
     <t>Chapel Photoshoot</t>
   </si>
   <si>
-    <t>[Photographer] 16:10~16:30 chapel photoshoot — then couple rests</t>
+    <t>16:10~16:30 chapel photoshoot — then couple rests</t>
   </si>
   <si>
     <t>16:35</t>
@@ -115,7 +115,7 @@
     <t>MC Preparation &amp; BGM Confirm</t>
   </si>
   <si>
-    <t>[MC] 16:00 MC spare check / 16:30 MC confirm BGM. Confirm Type-C BGM for opening slideshow &amp; entrance.</t>
+    <t>16:00 MC spare check / 16:30 MC confirm BGM. Confirm Type-C BGM for opening slideshow &amp; entrance.</t>
   </si>
   <si>
     <t>16:50</t>
@@ -124,16 +124,13 @@
     <t>Waiting for Entrance</t>
   </si>
   <si>
-    <t>[Couple]</t>
-  </si>
-  <si>
     <t>17:00</t>
   </si>
   <si>
     <t>Slideshow</t>
   </si>
   <si>
-    <t>[Tech] BGM: Type-C. Slideshow of couple's lifestyle photos &amp; highlight video — plays before entrance begins.</t>
+    <t>BGM: Type-C. Slideshow of couple's lifestyle photos &amp; highlight video — plays before entrance begins.</t>
   </si>
   <si>
     <t>① Type-C</t>
@@ -145,7 +142,7 @@
     <t>Groom Entrance with Friends 🎭</t>
   </si>
   <si>
-    <t>[Groom] BGM: Type-C entrance. Groom enters with friends one by one → waits at centre of floor.</t>
+    <t>BGM: Type-C entrance. Groom enters with friends one by one → waits at centre of floor.</t>
   </si>
   <si>
     <t>② Groom Entrance BGM (Type-C)</t>
@@ -157,7 +154,7 @@
     <t>Bride Entrance with Father — Handover 🎭</t>
   </si>
   <si>
-    <t>[Bride] Bride enters with father → father handover to groom</t>
+    <t>Bride enters with father → father handover to groom</t>
   </si>
   <si>
     <t>③ Bride Entrance BGM</t>
@@ -178,7 +175,7 @@
     <t>Ceremony 🎤 🎭</t>
   </si>
   <si>
-    <t>[MC] 15 min. Tint Htoo Aung (groom) has active role. Mg Mg Phyo officiating — 3 people on stage.</t>
+    <t>15 min. Tint Htoo Aung (groom) has active role. Mg Mg Phyo officiating — 3 people on stage.</t>
   </si>
   <si>
     <t>17:35</t>
@@ -187,7 +184,7 @@
     <t>Kanpai — Welcome Toast 🎤 🎭</t>
   </si>
   <si>
-    <t>[Guest (Friend)] Friend (Mg Mg Phyo) gives welcome speech → Kanpai toast.</t>
+    <t>Friend (Mg Mg Phyo) gives welcome speech → Kanpai toast.</t>
   </si>
   <si>
     <t>17:40</t>
@@ -196,7 +193,7 @@
     <t>Cake Cutting — First Bite, First Kiss &amp; Rings 🎭</t>
   </si>
   <si>
-    <t>[Couple] Sequence (venue confirmed): Cake cutting → First bite (groom feeds bride) → Ring reveal to guests → First kiss.</t>
+    <t>Sequence (venue confirmed): Cake cutting → First bite (groom feeds bride) → Ring reveal to guests → First kiss.</t>
   </si>
   <si>
     <t>⑤ Cake BGM</t>
@@ -208,7 +205,7 @@
     <t>Couple Exit — Flash Phone Lights 🎭</t>
   </si>
   <si>
-    <t>[Couple] Guests hold up phone flashlights to send off couple for costume change. Groom's 2nd outfit: T-shirt + coat.</t>
+    <t>Guests hold up phone flashlights to send off couple for costume change. Groom's 2nd outfit: T-shirt + coat.</t>
   </si>
   <si>
     <t>17:55</t>
@@ -217,7 +214,7 @@
     <t>Chuza Entertainment — Game Paper, Glow Sticks &amp; AI Movie</t>
   </si>
   <si>
-    <t>[MC / Tech] Distribute game quiz paper + glow sticks to ALL guests. AI/profile video plays simultaneously. Photographer takes table photos during this time.</t>
+    <t>Distribute game quiz paper + glow sticks to ALL guests. AI/profile video plays simultaneously. Photographer takes table photos during this time.</t>
   </si>
   <si>
     <t>18:10</t>
@@ -226,7 +223,7 @@
     <t>Re-entrance — Laser Show, Stairs &amp; Love Speech 🎭</t>
   </si>
   <si>
-    <t>[Couple] Laser show → couple descends from 2F Gallery stairs → Love speech (guests hold lit glow sticks). BGM: Sweet Heart.</t>
+    <t>Laser show → couple descends from 2F Gallery stairs → Love speech (guests hold lit glow sticks). BGM: Sweet Heart.</t>
   </si>
   <si>
     <t>⑥ Sweet Heart</t>
@@ -238,7 +235,7 @@
     <t>Guest Speeches — Father &amp; Friends 🎤 🎭</t>
   </si>
   <si>
-    <t>[Guest (Father / Friend)] 1–2 groups (father's side + friend's side). Each group within 5 min. MC to introduce each speaker. Couple stands at front of stage.</t>
+    <t>1–2 groups (father's side + friend's side). Each group within 5 min. MC to introduce each speaker. Couple stands at front of stage.</t>
   </si>
   <si>
     <t>18:30</t>
@@ -247,7 +244,7 @@
     <t>Game — MC Quiz 🎤 🎭</t>
   </si>
   <si>
-    <t>[MC] 10 questions about the couple (use the game paper distributed during 中座). Guests with 5+ correct answers win a prize — couple provides prizes. Confirm rehearsal &amp; sound check with MC.</t>
+    <t>10 questions about the couple (use the game paper distributed during 中座). Guests with 5+ correct answers win a prize — couple provides prizes. Confirm rehearsal &amp; sound check with MC.</t>
   </si>
   <si>
     <t>18:45</t>
@@ -256,7 +253,7 @@
     <t>Round Table Photo</t>
   </si>
   <si>
-    <t>[Couple / Photo] Couple visits each table for photos. Table layout: approx. 10 round tables × 30 guests / 9 round tables × 36 guests. Photographer covers all tables.</t>
+    <t>Couple visits each table for photos. Table layout: approx. 10 round tables × 30 guests / 9 round tables × 36 guests. Photographer covers all tables.</t>
   </si>
   <si>
     <t>19:00</t>
@@ -265,7 +262,7 @@
     <t>Letter to Family — Bride 🎤 🎭</t>
   </si>
   <si>
-    <t>[Bride] Bride reads letter to family with soft backing BGM. Tech: cue music at the start. Tissues ready.</t>
+    <t>Bride reads letter to family with soft backing BGM. Tech: cue music at the start. Tissues ready.</t>
   </si>
   <si>
     <t>19:05</t>
@@ -274,16 +271,13 @@
     <t>Thank You Message — Groom 🎤 🎭</t>
   </si>
   <si>
-    <t>[Groom]</t>
-  </si>
-  <si>
     <t>19:10</t>
   </si>
   <si>
     <t>Flower Shower 🎭</t>
   </si>
   <si>
-    <t>[Guests] Key highlight moment. Couple walks through flower shower from guests.</t>
+    <t>Key highlight moment. Couple walks through flower shower from guests.</t>
   </si>
   <si>
     <t>⑦ Flower Shower BGM</t>
@@ -295,7 +289,7 @@
     <t>Bouquet Toss from Stairs 🎭</t>
   </si>
   <si>
-    <t>[Bride] Bride throws bouquet from top of 2F Gallery stairs down to guests at ground floor.</t>
+    <t>Bride throws bouquet from top of 2F Gallery stairs down to guests at ground floor.</t>
   </si>
   <si>
     <t>19:25</t>
@@ -304,7 +298,7 @@
     <t>Group Photo</t>
   </si>
   <si>
-    <t>[Photographer] All guests + couple + family. Photographer coordinates positioning.</t>
+    <t>All guests + couple + family. Photographer coordinates positioning.</t>
   </si>
   <si>
     <t>19:35</t>
@@ -313,7 +307,7 @@
     <t>Depart — Both Together 🎭</t>
   </si>
   <si>
-    <t>[Couple] Both exit together through 1 door. Guests line both sides and applaud/wave.</t>
+    <t>Both exit together through 1 door. Guests line both sides and applaud/wave.</t>
   </si>
   <si>
     <t>⑧ Departure BGM</t>
@@ -325,7 +319,7 @@
     <t>Lobby — Petit Gift Farewell</t>
   </si>
   <si>
-    <t>[Couple] Couple stands at lobby entrance, gives petit gift to each departing guest. Photographer captures farewell moments. Party closes at 19:30.</t>
+    <t>Couple stands at lobby entrance, gives petit gift to each departing guest. Photographer captures farewell moments. Party closes at 19:30.</t>
   </si>
 </sst>
 </file>
@@ -1170,7 +1164,7 @@
         <v>24</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F13" s="24"/>
       <c r="G13" s="24"/>
@@ -1181,101 +1175,101 @@
     </row>
     <row r="14" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="24" t="s">
         <v>39</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>40</v>
       </c>
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I14" s="25"/>
     </row>
     <row r="15" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="24" t="s">
         <v>43</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="24" t="s">
-        <v>44</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="24"/>
       <c r="H15" s="25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I15" s="25"/>
     </row>
     <row r="16" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="24" t="s">
         <v>47</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="24" t="s">
-        <v>48</v>
       </c>
       <c r="F16" s="24"/>
       <c r="G16" s="24"/>
       <c r="H16" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I16" s="25"/>
     </row>
     <row r="17" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D17" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F17" s="24"/>
       <c r="G17" s="24"/>
       <c r="H17" s="25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I17" s="25"/>
     </row>
     <row r="18" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="24" t="s">
         <v>54</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>55</v>
       </c>
       <c r="F18" s="24"/>
       <c r="G18" s="24"/>
@@ -1286,17 +1280,17 @@
     </row>
     <row r="19" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B19" s="21"/>
       <c r="C19" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="24" t="s">
         <v>57</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>58</v>
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
@@ -1307,38 +1301,38 @@
     </row>
     <row r="20" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B20" s="21"/>
       <c r="C20" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="24" t="s">
         <v>60</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="24" t="s">
-        <v>61</v>
       </c>
       <c r="F20" s="24"/>
       <c r="G20" s="24"/>
       <c r="H20" s="25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I20" s="25"/>
     </row>
     <row r="21" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" s="21"/>
       <c r="C21" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="24" t="s">
         <v>64</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E21" s="24" t="s">
-        <v>65</v>
       </c>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
@@ -1349,17 +1343,17 @@
     </row>
     <row r="22" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="24" t="s">
         <v>67</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E22" s="24" t="s">
-        <v>68</v>
       </c>
       <c r="F22" s="24"/>
       <c r="G22" s="24"/>
@@ -1370,38 +1364,38 @@
     </row>
     <row r="23" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B23" s="21"/>
       <c r="C23" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="24" t="s">
         <v>70</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="24" t="s">
-        <v>71</v>
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
       <c r="H23" s="25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I23" s="25"/>
     </row>
     <row r="24" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="24" t="s">
         <v>74</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" s="24" t="s">
-        <v>75</v>
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
@@ -1412,17 +1406,17 @@
     </row>
     <row r="25" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B25" s="21"/>
       <c r="C25" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E25" s="24" t="s">
         <v>77</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E25" s="24" t="s">
-        <v>78</v>
       </c>
       <c r="F25" s="24"/>
       <c r="G25" s="24"/>
@@ -1433,17 +1427,17 @@
     </row>
     <row r="26" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B26" s="21"/>
       <c r="C26" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="24" t="s">
         <v>80</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="24" t="s">
-        <v>81</v>
       </c>
       <c r="F26" s="24"/>
       <c r="G26" s="24"/>
@@ -1454,17 +1448,17 @@
     </row>
     <row r="27" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" s="21"/>
       <c r="C27" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" s="24" t="s">
         <v>83</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="E27" s="24" t="s">
-        <v>84</v>
       </c>
       <c r="F27" s="24"/>
       <c r="G27" s="24"/>
@@ -1475,17 +1469,17 @@
     </row>
     <row r="28" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D28" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
@@ -1496,38 +1490,38 @@
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="26" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D29" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
       <c r="H29" s="25" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="I29" s="25"/>
     </row>
     <row r="30" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B30" s="21"/>
       <c r="C30" s="26" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D30" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E30" s="24" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F30" s="24"/>
       <c r="G30" s="24"/>
@@ -1538,17 +1532,17 @@
     </row>
     <row r="31" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B31" s="21"/>
       <c r="C31" s="26" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D31" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E31" s="24" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F31" s="24"/>
       <c r="G31" s="24"/>
@@ -1559,38 +1553,38 @@
     </row>
     <row r="32" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B32" s="21"/>
       <c r="C32" s="26" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D32" s="23" t="s">
         <v>24</v>
       </c>
       <c r="E32" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F32" s="24"/>
       <c r="G32" s="24"/>
       <c r="H32" s="25" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I32" s="25"/>
     </row>
     <row r="33" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B33" s="27"/>
       <c r="C33" s="28" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D33" s="16" t="s">
         <v>24</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F33" s="29"/>
       <c r="G33" s="29"/>

</xml_diff>

<commit_message>
Add location and coordinationNotesJa to all Louis Htoo plan activities
All 20 activities in 2026-06-21-LouisHtoo.json now have:
- location field (ロビー, 2F, チャペル, ステージ, バージンロード, 各テーブル, etc.)
- coordinationNotesJa (Japanese translation of all coordination notes)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="117">
   <si>
     <t>Hotel Bell Classic_WEDDING PARTY PLAN</t>
   </si>
@@ -85,18 +85,24 @@
     <t>Guest Reception</t>
   </si>
   <si>
+    <t>ロビー</t>
+  </si>
+  <si>
+    <t>15:30 First meet — Video &amp; Photo team on standby. Venue setup: banner posters, tent cards, small tables, DMC QR code cards at each seat.</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>15:30 First meet — Video &amp; Photo team on standby. Venue setup: banner posters, tent cards, small tables, DMC QR code cards at each seat.</t>
-  </si>
-  <si>
     <t>15:50</t>
   </si>
   <si>
     <t>Group Photo 2F</t>
   </si>
   <si>
+    <t>2F</t>
+  </si>
+  <si>
     <t>15:45 — 2F group photo with guests</t>
   </si>
   <si>
@@ -106,6 +112,9 @@
     <t>Chapel Photoshoot</t>
   </si>
   <si>
+    <t>チャペル</t>
+  </si>
+  <si>
     <t>16:10~16:30 chapel photoshoot — then couple rests</t>
   </si>
   <si>
@@ -115,6 +124,9 @@
     <t>MC Preparation &amp; BGM Confirm</t>
   </si>
   <si>
+    <t>会場内</t>
+  </si>
+  <si>
     <t>16:00 MC spare check / 16:30 MC confirm BGM. Confirm Type-C BGM for opening slideshow &amp; entrance.</t>
   </si>
   <si>
@@ -124,12 +136,18 @@
     <t>Waiting for Entrance</t>
   </si>
   <si>
+    <t>バックステージ</t>
+  </si>
+  <si>
     <t>17:00</t>
   </si>
   <si>
     <t>Slideshow</t>
   </si>
   <si>
+    <t>会場（スクリーン）</t>
+  </si>
+  <si>
     <t>BGM: Type-C. Slideshow of couple's lifestyle photos &amp; highlight video — plays before entrance begins.</t>
   </si>
   <si>
@@ -142,6 +160,9 @@
     <t>Groom Entrance with Friends 🎭</t>
   </si>
   <si>
+    <t>1F 会場</t>
+  </si>
+  <si>
     <t>BGM: Type-C entrance. Groom enters with friends one by one → waits at centre of floor.</t>
   </si>
   <si>
@@ -154,6 +175,9 @@
     <t>Bride Entrance with Father — Handover 🎭</t>
   </si>
   <si>
+    <t>バージンロード</t>
+  </si>
+  <si>
     <t>Bride enters with father → father handover to groom</t>
   </si>
   <si>
@@ -175,6 +199,9 @@
     <t>Ceremony 🎤 🎭</t>
   </si>
   <si>
+    <t>ステージ</t>
+  </si>
+  <si>
     <t>15 min. Tint Htoo Aung (groom) has active role. Mg Mg Phyo officiating — 3 people on stage.</t>
   </si>
   <si>
@@ -214,6 +241,9 @@
     <t>Chuza Entertainment — Game Paper, Glow Sticks &amp; AI Movie</t>
   </si>
   <si>
+    <t>会場</t>
+  </si>
+  <si>
     <t>Distribute game quiz paper + glow sticks to ALL guests. AI/profile video plays simultaneously. Photographer takes table photos during this time.</t>
   </si>
   <si>
@@ -223,6 +253,9 @@
     <t>Re-entrance — Laser Show, Stairs &amp; Love Speech 🎭</t>
   </si>
   <si>
+    <t>2F ギャラリー</t>
+  </si>
+  <si>
     <t>Laser show → couple descends from 2F Gallery stairs → Love speech (guests hold lit glow sticks). BGM: Sweet Heart.</t>
   </si>
   <si>
@@ -253,6 +286,9 @@
     <t>Round Table Photo</t>
   </si>
   <si>
+    <t>各テーブル</t>
+  </si>
+  <si>
     <t>Couple visits each table for photos. Table layout: approx. 10 round tables × 30 guests / 9 round tables × 36 guests. Photographer covers all tables.</t>
   </si>
   <si>
@@ -289,6 +325,9 @@
     <t>Bouquet Toss from Stairs 🎭</t>
   </si>
   <si>
+    <t>2F 階段</t>
+  </si>
+  <si>
     <t>Bride throws bouquet from top of 2F Gallery stairs down to guests at ground floor.</t>
   </si>
   <si>
@@ -305,6 +344,9 @@
   </si>
   <si>
     <t>Depart — Both Together 🎭</t>
+  </si>
+  <si>
+    <t>1F 出口</t>
   </si>
   <si>
     <t>Both exit together through 1 door. Guests line both sides and applaud/wave.</t>
@@ -1085,511 +1127,511 @@
       <c r="F9" s="24"/>
       <c r="G9" s="24"/>
       <c r="H9" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I9" s="25"/>
     </row>
     <row r="10" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F10" s="24"/>
       <c r="G10" s="24"/>
       <c r="H10" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I10" s="25"/>
     </row>
     <row r="11" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="22" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F11" s="24"/>
       <c r="G11" s="24"/>
       <c r="H11" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I11" s="25"/>
     </row>
     <row r="12" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="22" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F12" s="24"/>
       <c r="G12" s="24"/>
       <c r="H12" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I12" s="25"/>
     </row>
     <row r="13" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="22" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F13" s="24"/>
       <c r="G13" s="24"/>
       <c r="H13" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I13" s="25"/>
     </row>
     <row r="14" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="26" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="25" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="I14" s="25"/>
     </row>
     <row r="15" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="26" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="24"/>
       <c r="H15" s="25" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="I15" s="25"/>
     </row>
     <row r="16" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="26" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F16" s="24"/>
       <c r="G16" s="24"/>
       <c r="H16" s="25" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="I16" s="25"/>
     </row>
     <row r="17" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="26" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F17" s="24"/>
       <c r="G17" s="24"/>
       <c r="H17" s="25" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I17" s="25"/>
     </row>
     <row r="18" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="26" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F18" s="24"/>
       <c r="G18" s="24"/>
       <c r="H18" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I18" s="25"/>
     </row>
     <row r="19" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B19" s="21"/>
       <c r="C19" s="26" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
       <c r="H19" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I19" s="25"/>
     </row>
     <row r="20" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B20" s="21"/>
       <c r="C20" s="26" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F20" s="24"/>
       <c r="G20" s="24"/>
       <c r="H20" s="25" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="I20" s="25"/>
     </row>
     <row r="21" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B21" s="21"/>
       <c r="C21" s="26" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
       <c r="H21" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I21" s="25"/>
     </row>
     <row r="22" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="26" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F22" s="24"/>
       <c r="G22" s="24"/>
       <c r="H22" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I22" s="25"/>
     </row>
     <row r="23" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="B23" s="21"/>
       <c r="C23" s="26" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
       <c r="H23" s="25" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="I23" s="25"/>
     </row>
     <row r="24" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="26" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
       <c r="H24" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I24" s="25"/>
     </row>
     <row r="25" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="B25" s="21"/>
       <c r="C25" s="26" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="F25" s="24"/>
       <c r="G25" s="24"/>
       <c r="H25" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I25" s="25"/>
     </row>
     <row r="26" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B26" s="21"/>
       <c r="C26" s="26" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>24</v>
+        <v>91</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="F26" s="24"/>
       <c r="G26" s="24"/>
       <c r="H26" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I26" s="25"/>
     </row>
     <row r="27" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="B27" s="21"/>
       <c r="C27" s="26" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="F27" s="24"/>
       <c r="G27" s="24"/>
       <c r="H27" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I27" s="25"/>
     </row>
     <row r="28" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="26" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
       <c r="H28" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I28" s="25"/>
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="26" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
       <c r="H29" s="25" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="I29" s="25"/>
     </row>
     <row r="30" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B30" s="21"/>
       <c r="C30" s="26" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>24</v>
+        <v>104</v>
       </c>
       <c r="E30" s="24" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="F30" s="24"/>
       <c r="G30" s="24"/>
       <c r="H30" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I30" s="25"/>
     </row>
     <row r="31" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B31" s="21"/>
       <c r="C31" s="26" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="E31" s="24" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="F31" s="24"/>
       <c r="G31" s="24"/>
       <c r="H31" s="25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I31" s="25"/>
     </row>
     <row r="32" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="B32" s="21"/>
       <c r="C32" s="26" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>24</v>
+        <v>111</v>
       </c>
       <c r="E32" s="24" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="F32" s="24"/>
       <c r="G32" s="24"/>
       <c r="H32" s="25" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="I32" s="25"/>
     </row>
     <row r="33" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="B33" s="27"/>
       <c r="C33" s="28" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D33" s="16" t="s">
         <v>24</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="F33" s="29"/>
       <c r="G33" s="29"/>
       <c r="H33" s="30" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I33" s="30"/>
     </row>

</xml_diff>

<commit_message>
Add role-specific staff notes (MC / Photo / Lighting) per activity
- Added staffNotes: { mc?, photo?, lighting? } field to Activity and TimelineActivity types
- Excel: staff notes render as color-coded sub-rows below each activity
  - 🎤 MC notes = light blue (FFD6EAF8)
  - 📸 Photo/Video notes = light orange (FFFDE8D8)
  - 💡 Lighting notes = light yellow (FFFEF9E7)
- UI: collapsible "Staff Notes" panel per timeline item with labeled textareas per role
- Louis Htoo plan: added staffNotes to 8 key activities (entrances, ceremony,
  cake cutting, re-entrance, letter to family, flower shower, bouquet toss)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="142">
   <si>
     <t>Hotel Bell Classic_WEDDING PARTY PLAN</t>
   </si>
@@ -169,6 +169,24 @@
     <t>② Groom Entrance BGM (Type-C)</t>
   </si>
   <si>
+    <t>🎤 MC</t>
+  </si>
+  <si>
+    <t>Announce groom's entrance with energy. Wait for groom to reach centre floor before moving on.</t>
+  </si>
+  <si>
+    <t>📸 Photo/Video</t>
+  </si>
+  <si>
+    <t>Position at 1F entrance. Capture groom walking in with friends — wide group shot then close-up on groom's face. VTR rolling.</t>
+  </si>
+  <si>
+    <t>💡 Lighting</t>
+  </si>
+  <si>
+    <t>Spotlight tracking groom from entrance to centre floor. Dim main hall for dramatic effect.</t>
+  </si>
+  <si>
     <t>17:10</t>
   </si>
   <si>
@@ -184,6 +202,15 @@
     <t>③ Bride Entrance BGM</t>
   </si>
   <si>
+    <t>Pause and give space at father handover — do not rush this moment.</t>
+  </si>
+  <si>
+    <t>One photographer at end of Virgin Road (stage side). Key shot: father's expression at handover. VTR: capture full walk.</t>
+  </si>
+  <si>
+    <t>Warm spotlight tracking bride from entrance to stage.</t>
+  </si>
+  <si>
     <t>17:15</t>
   </si>
   <si>
@@ -205,6 +232,15 @@
     <t>15 min. Tint Htoo Aung (groom) has active role. Mg Mg Phyo officiating — 3 people on stage.</t>
   </si>
   <si>
+    <t>Groom (Tint Htoo Aung) has an active speaking role — confirm his cues beforehand. Officiant: Mg Mg Phyo.</t>
+  </si>
+  <si>
+    <t>Cover: officiant, couple's expressions, and any ring/vow moment close-ups. VTR rolling throughout. 3 people on stage.</t>
+  </si>
+  <si>
+    <t>Steady, bright, even lighting throughout ceremony. No dramatic changes.</t>
+  </si>
+  <si>
     <t>17:35</t>
   </si>
   <si>
@@ -226,6 +262,15 @@
     <t>⑤ Cake BGM</t>
   </si>
   <si>
+    <t>Narrate each step and build anticipation. Count down before first kiss.</t>
+  </si>
+  <si>
+    <t>4 key shots in sequence: (1) knife on cake, (2) first bite — get both faces, (3) ring reveal — shoot from above/front, (4) first kiss. Do NOT miss ring reveal!</t>
+  </si>
+  <si>
+    <t>Bright stage lighting. Flash-friendly.</t>
+  </si>
+  <si>
     <t>17:50</t>
   </si>
   <si>
@@ -262,6 +307,15 @@
     <t>⑥ Sweet Heart</t>
   </si>
   <si>
+    <t>Build crowd energy before laser show starts. Cue music (Sweet Heart). Let love speech breathe — do not interrupt.</t>
+  </si>
+  <si>
+    <t>VTR: wide shot from 2F showing laser show + staircase descent. Snapshot: couple's faces + full crowd with glowing sticks.</t>
+  </si>
+  <si>
+    <t>Laser show sequence on cue. After descent, transition to warm romantic lighting for love speech.</t>
+  </si>
+  <si>
     <t>18:20</t>
   </si>
   <si>
@@ -301,6 +355,15 @@
     <t>Bride reads letter to family with soft backing BGM. Tech: cue music at the start. Tissues ready.</t>
   </si>
   <si>
+    <t>Stand by but remain silent. Cue backing BGM softly at the start of reading.</t>
+  </si>
+  <si>
+    <t>Capture bride reading + family members' reactions. Be discreet — no flash. VTR: steady wide shot.</t>
+  </si>
+  <si>
+    <t>Soft warm lighting only. Reduce brightness.</t>
+  </si>
+  <si>
     <t>19:05</t>
   </si>
   <si>
@@ -319,6 +382,12 @@
     <t>⑦ Flower Shower BGM</t>
   </si>
   <si>
+    <t>Wide shot of full shower + close-up of couple's faces. VTR: overhead angle if possible. This is a key highlight moment.</t>
+  </si>
+  <si>
+    <t>Full bright warm lighting — joyful and celebratory.</t>
+  </si>
+  <si>
     <t>19:15</t>
   </si>
   <si>
@@ -329,6 +398,12 @@
   </si>
   <si>
     <t>Bride throws bouquet from top of 2F Gallery stairs down to guests at ground floor.</t>
+  </si>
+  <si>
+    <t>Gather single women to the floor. Build excitement with countdown.</t>
+  </si>
+  <si>
+    <t>Split: one photographer on stairs with bride, one in crowd below. Capture the toss arc + catch moment.</t>
   </si>
   <si>
     <t>19:25</t>
@@ -368,7 +443,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -412,8 +487,18 @@
       <color rgb="FF888888"/>
       <name val="MS P Mincho"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="MS P Mincho"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <name val="MS P Mincho"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -428,6 +513,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDE8D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF9E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -555,7 +655,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -622,6 +722,30 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -974,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="8" style="1" customWidth="1"/>
@@ -1257,187 +1381,163 @@
       </c>
       <c r="I15" s="25"/>
     </row>
-    <row r="16" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
+    <row r="16" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="27"/>
+      <c r="C16" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="26" t="s">
+      <c r="D16" s="29"/>
+      <c r="E16" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="31"/>
+      <c r="C17" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="D17" s="33"/>
+      <c r="E17" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="25" t="s">
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="35"/>
+      <c r="C18" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="I16" s="25"/>
-    </row>
-    <row r="17" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
+      <c r="D18" s="37"/>
+      <c r="E18" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17" s="25"/>
-    </row>
-    <row r="18" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I18" s="25"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
     </row>
     <row r="19" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B19" s="21"/>
       <c r="C19" s="26" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
       <c r="H19" s="25" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="I19" s="25"/>
     </row>
-    <row r="20" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="I20" s="25"/>
-    </row>
-    <row r="21" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E21" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I21" s="25"/>
-    </row>
-    <row r="22" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="E22" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I22" s="25"/>
+    <row r="20" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="27"/>
+      <c r="C20" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="29"/>
+      <c r="E20" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="31"/>
+      <c r="C21" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="33"/>
+      <c r="E21" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="35"/>
+      <c r="C22" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="37"/>
+      <c r="E22" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="38"/>
     </row>
     <row r="23" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="B23" s="21"/>
       <c r="C23" s="26" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
       <c r="H23" s="25" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="I23" s="25"/>
     </row>
     <row r="24" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="B24" s="21"/>
       <c r="C24" s="26" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
@@ -1446,82 +1546,70 @@
       </c>
       <c r="I24" s="25"/>
     </row>
-    <row r="25" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="E25" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I25" s="25"/>
-    </row>
-    <row r="26" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="E26" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I26" s="25"/>
-    </row>
-    <row r="27" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="B27" s="21"/>
-      <c r="C27" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I27" s="25"/>
+    <row r="25" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="27"/>
+      <c r="C25" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="29"/>
+      <c r="E25" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="31"/>
+      <c r="C26" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="33"/>
+      <c r="E26" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="35"/>
+      <c r="C27" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="37"/>
+      <c r="E27" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
     </row>
     <row r="28" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="26" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
@@ -1532,111 +1620,521 @@
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="26" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
       <c r="H29" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="I29" s="25"/>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" s="27"/>
+      <c r="C30" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="29"/>
+      <c r="E30" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="31"/>
+      <c r="C31" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="33"/>
+      <c r="E31" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="35"/>
+      <c r="C32" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" s="37"/>
+      <c r="E32" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
+    </row>
+    <row r="33" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="21"/>
+      <c r="C33" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I33" s="25"/>
+    </row>
+    <row r="34" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="21"/>
+      <c r="C34" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I34" s="25"/>
+    </row>
+    <row r="35" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" s="21"/>
+      <c r="C35" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="E35" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="I35" s="25"/>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36" s="27"/>
+      <c r="C36" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" s="29"/>
+      <c r="E36" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="30"/>
+    </row>
+    <row r="37" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" s="31"/>
+      <c r="C37" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D37" s="33"/>
+      <c r="E37" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="34"/>
+      <c r="I37" s="34"/>
+    </row>
+    <row r="38" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38" s="35"/>
+      <c r="C38" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" s="37"/>
+      <c r="E38" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+    </row>
+    <row r="39" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="I29" s="25"/>
-    </row>
-    <row r="30" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="21" t="s">
+      <c r="B39" s="21"/>
+      <c r="C39" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="26" t="s">
+      <c r="D39" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E39" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="D30" s="23" t="s">
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I39" s="25"/>
+    </row>
+    <row r="40" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="E30" s="24" t="s">
+      <c r="B40" s="21"/>
+      <c r="C40" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I30" s="25"/>
-    </row>
-    <row r="31" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="21" t="s">
+      <c r="D40" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E40" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="26" t="s">
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I40" s="25"/>
+    </row>
+    <row r="41" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="D31" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="E31" s="24" t="s">
+      <c r="B41" s="21"/>
+      <c r="C41" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I31" s="25"/>
-    </row>
-    <row r="32" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="21" t="s">
+      <c r="D41" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="B32" s="21"/>
-      <c r="C32" s="26" t="s">
+      <c r="E41" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="F41" s="24"/>
+      <c r="G41" s="24"/>
+      <c r="H41" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I41" s="25"/>
+    </row>
+    <row r="42" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="B42" s="21"/>
+      <c r="C42" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="25" t="s">
+      <c r="D42" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E42" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="I32" s="25"/>
-    </row>
-    <row r="33" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I42" s="25"/>
+    </row>
+    <row r="43" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B43" s="27"/>
+      <c r="C43" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D43" s="29"/>
+      <c r="E43" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="28" t="s">
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="30"/>
+    </row>
+    <row r="44" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" s="31"/>
+      <c r="C44" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D44" s="33"/>
+      <c r="E44" s="34" t="s">
         <v>115</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="F44" s="34"/>
+      <c r="G44" s="34"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="34"/>
+    </row>
+    <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B45" s="35"/>
+      <c r="C45" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38" t="s">
+        <v>116</v>
+      </c>
+      <c r="F45" s="38"/>
+      <c r="G45" s="38"/>
+      <c r="H45" s="38"/>
+      <c r="I45" s="38"/>
+    </row>
+    <row r="46" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" s="21"/>
+      <c r="C46" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="D46" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="F46" s="24"/>
+      <c r="G46" s="24"/>
+      <c r="H46" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I46" s="25"/>
+    </row>
+    <row r="47" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" s="21"/>
+      <c r="C47" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E47" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="F47" s="24"/>
+      <c r="G47" s="24"/>
+      <c r="H47" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="I47" s="25"/>
+    </row>
+    <row r="48" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B48" s="31"/>
+      <c r="C48" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D48" s="33"/>
+      <c r="E48" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="F48" s="34"/>
+      <c r="G48" s="34"/>
+      <c r="H48" s="34"/>
+      <c r="I48" s="34"/>
+    </row>
+    <row r="49" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B49" s="35"/>
+      <c r="C49" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="D49" s="37"/>
+      <c r="E49" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="F49" s="38"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="38"/>
+    </row>
+    <row r="50" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B50" s="21"/>
+      <c r="C50" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="D50" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="E50" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="F50" s="24"/>
+      <c r="G50" s="24"/>
+      <c r="H50" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I50" s="25"/>
+    </row>
+    <row r="51" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B51" s="27"/>
+      <c r="C51" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="D51" s="29"/>
+      <c r="E51" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
+      <c r="I51" s="30"/>
+    </row>
+    <row r="52" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B52" s="31"/>
+      <c r="C52" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D52" s="33"/>
+      <c r="E52" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="F52" s="34"/>
+      <c r="G52" s="34"/>
+      <c r="H52" s="34"/>
+      <c r="I52" s="34"/>
+    </row>
+    <row r="53" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="B53" s="21"/>
+      <c r="C53" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="D53" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="E53" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="F53" s="24"/>
+      <c r="G53" s="24"/>
+      <c r="H53" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I53" s="25"/>
+    </row>
+    <row r="54" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="B54" s="21"/>
+      <c r="C54" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="D54" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="E54" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="F54" s="24"/>
+      <c r="G54" s="24"/>
+      <c r="H54" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="I54" s="25"/>
+    </row>
+    <row r="55" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="39" t="s">
+        <v>139</v>
+      </c>
+      <c r="B55" s="39"/>
+      <c r="C55" s="40" t="s">
+        <v>140</v>
+      </c>
+      <c r="D55" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E33" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="I33" s="30"/>
+      <c r="E55" s="41" t="s">
+        <v>141</v>
+      </c>
+      <c r="F55" s="41"/>
+      <c r="G55" s="41"/>
+      <c r="H55" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="I55" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="90">
+  <mergeCells count="134">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:D4"/>
     <mergeCell ref="F2:G2"/>
@@ -1674,26 +2172,20 @@
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="E16:I16"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="E17:I17"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="E18:I18"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="E20:I20"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="E21:I21"/>
     <mergeCell ref="A22:B22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="E22:I22"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:I23"/>
@@ -1701,14 +2193,11 @@
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="A25:B25"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="E25:I25"/>
     <mergeCell ref="A26:B26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="E26:I26"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="E27:I27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="E28:G28"/>
     <mergeCell ref="H28:I28"/>
@@ -1716,17 +2205,70 @@
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="A30:B30"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="E30:I30"/>
     <mergeCell ref="A31:B31"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="E31:I31"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="E32:I32"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="E33:G33"/>
     <mergeCell ref="H33:I33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="E40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="E42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="E43:I43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="E44:I44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="E48:I48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="E49:I49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="E51:I51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="E52:I52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="H55:I55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Add スタッフ column (J) with stacked MC/Photo/Lighting notes in Excel
Replaces the previous 3-sub-row approach with a single compact column J
showing 🎤/📸/💡 icon lines per activity row. Row height auto-scales
based on number of staff note lines. Applied to both browser generator
(excelGenerator.ts) and server-side generator (generate-excel.cjs).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011b8G8QVWKtuGUgUNDGjwyR
</commit_message>
<xml_diff>
--- a/Wedding_Plan_20260621_Louis_Htoo.xlsx
+++ b/Wedding_Plan_20260621_Louis_Htoo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="126">
   <si>
     <t>Hotel Bell Classic_WEDDING PARTY PLAN</t>
   </si>
@@ -79,6 +79,9 @@
     <t>BGM</t>
   </si>
   <si>
+    <t>スタッフ</t>
+  </si>
+  <si>
     <t>15:20</t>
   </si>
   <si>
@@ -169,22 +172,9 @@
     <t>② Groom Entrance BGM (Type-C)</t>
   </si>
   <si>
-    <t>🎤 MC</t>
-  </si>
-  <si>
-    <t>Announce groom's entrance with energy. Wait for groom to reach centre floor before moving on.</t>
-  </si>
-  <si>
-    <t>📸 Photo/Video</t>
-  </si>
-  <si>
-    <t>Position at 1F entrance. Capture groom walking in with friends — wide group shot then close-up on groom's face. VTR rolling.</t>
-  </si>
-  <si>
-    <t>💡 Lighting</t>
-  </si>
-  <si>
-    <t>Spotlight tracking groom from entrance to centre floor. Dim main hall for dramatic effect.</t>
+    <t xml:space="preserve">🎤 Announce groom's entrance with energy. Wait for groom to reach centre floor before moving on.
+📸 Position at 1F entrance. Capture groom walking in with friends — wide group shot then close-up on groom's face. VTR rolling.
+💡 Spotlight tracking groom from entrance to centre floor. Dim main hall for dramatic effect.</t>
   </si>
   <si>
     <t>17:10</t>
@@ -202,13 +192,9 @@
     <t>③ Bride Entrance BGM</t>
   </si>
   <si>
-    <t>Pause and give space at father handover — do not rush this moment.</t>
-  </si>
-  <si>
-    <t>One photographer at end of Virgin Road (stage side). Key shot: father's expression at handover. VTR: capture full walk.</t>
-  </si>
-  <si>
-    <t>Warm spotlight tracking bride from entrance to stage.</t>
+    <t xml:space="preserve">🎤 Pause and give space at father handover — do not rush this moment.
+📸 One photographer at end of Virgin Road (stage side). Key shot: father's expression at handover. VTR: capture full walk.
+💡 Warm spotlight tracking bride from entrance to stage.</t>
   </si>
   <si>
     <t>17:15</t>
@@ -232,13 +218,9 @@
     <t>15 min. Tint Htoo Aung (groom) has active role. Mg Mg Phyo officiating — 3 people on stage.</t>
   </si>
   <si>
-    <t>Groom (Tint Htoo Aung) has an active speaking role — confirm his cues beforehand. Officiant: Mg Mg Phyo.</t>
-  </si>
-  <si>
-    <t>Cover: officiant, couple's expressions, and any ring/vow moment close-ups. VTR rolling throughout. 3 people on stage.</t>
-  </si>
-  <si>
-    <t>Steady, bright, even lighting throughout ceremony. No dramatic changes.</t>
+    <t xml:space="preserve">🎤 Groom (Tint Htoo Aung) has an active speaking role — confirm his cues beforehand. Officiant: Mg Mg Phyo.
+📸 Cover: officiant, couple's expressions, and any ring/vow moment close-ups. VTR rolling throughout. 3 people on stage.
+💡 Steady, bright, even lighting throughout ceremony. No dramatic changes.</t>
   </si>
   <si>
     <t>17:35</t>
@@ -262,13 +244,9 @@
     <t>⑤ Cake BGM</t>
   </si>
   <si>
-    <t>Narrate each step and build anticipation. Count down before first kiss.</t>
-  </si>
-  <si>
-    <t>4 key shots in sequence: (1) knife on cake, (2) first bite — get both faces, (3) ring reveal — shoot from above/front, (4) first kiss. Do NOT miss ring reveal!</t>
-  </si>
-  <si>
-    <t>Bright stage lighting. Flash-friendly.</t>
+    <t xml:space="preserve">🎤 Narrate each step and build anticipation. Count down before first kiss.
+📸 4 key shots in sequence: (1) knife on cake, (2) first bite — get both faces, (3) ring reveal — shoot from above/front, (4) first kiss. Do NOT miss ring reveal!
+💡 Bright stage lighting. Flash-friendly.</t>
   </si>
   <si>
     <t>17:50</t>
@@ -307,13 +285,9 @@
     <t>⑥ Sweet Heart</t>
   </si>
   <si>
-    <t>Build crowd energy before laser show starts. Cue music (Sweet Heart). Let love speech breathe — do not interrupt.</t>
-  </si>
-  <si>
-    <t>VTR: wide shot from 2F showing laser show + staircase descent. Snapshot: couple's faces + full crowd with glowing sticks.</t>
-  </si>
-  <si>
-    <t>Laser show sequence on cue. After descent, transition to warm romantic lighting for love speech.</t>
+    <t xml:space="preserve">🎤 Build crowd energy before laser show starts. Cue music (Sweet Heart). Let love speech breathe — do not interrupt.
+📸 VTR: wide shot from 2F showing laser show + staircase descent. Snapshot: couple's faces + full crowd with glowing sticks.
+💡 Laser show sequence on cue. After descent, transition to warm romantic lighting for love speech.</t>
   </si>
   <si>
     <t>18:20</t>
@@ -355,13 +329,9 @@
     <t>Bride reads letter to family with soft backing BGM. Tech: cue music at the start. Tissues ready.</t>
   </si>
   <si>
-    <t>Stand by but remain silent. Cue backing BGM softly at the start of reading.</t>
-  </si>
-  <si>
-    <t>Capture bride reading + family members' reactions. Be discreet — no flash. VTR: steady wide shot.</t>
-  </si>
-  <si>
-    <t>Soft warm lighting only. Reduce brightness.</t>
+    <t xml:space="preserve">🎤 Stand by but remain silent. Cue backing BGM softly at the start of reading.
+📸 Capture bride reading + family members' reactions. Be discreet — no flash. VTR: steady wide shot.
+💡 Soft warm lighting only. Reduce brightness.</t>
   </si>
   <si>
     <t>19:05</t>
@@ -382,10 +352,8 @@
     <t>⑦ Flower Shower BGM</t>
   </si>
   <si>
-    <t>Wide shot of full shower + close-up of couple's faces. VTR: overhead angle if possible. This is a key highlight moment.</t>
-  </si>
-  <si>
-    <t>Full bright warm lighting — joyful and celebratory.</t>
+    <t xml:space="preserve">📸 Wide shot of full shower + close-up of couple's faces. VTR: overhead angle if possible. This is a key highlight moment.
+💡 Full bright warm lighting — joyful and celebratory.</t>
   </si>
   <si>
     <t>19:15</t>
@@ -400,10 +368,8 @@
     <t>Bride throws bouquet from top of 2F Gallery stairs down to guests at ground floor.</t>
   </si>
   <si>
-    <t>Gather single women to the floor. Build excitement with countdown.</t>
-  </si>
-  <si>
-    <t>Split: one photographer on stairs with bride, one in crowd below. Capture the toss arc + catch moment.</t>
+    <t xml:space="preserve">🎤 Gather single women to the floor. Build excitement with countdown.
+📸 Split: one photographer on stairs with bride, one in crowd below. Capture the toss arc + catch moment.</t>
   </si>
   <si>
     <t>19:25</t>
@@ -443,7 +409,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -488,17 +454,11 @@
       <name val="MS P Mincho"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <name val="MS P Mincho"/>
-    </font>
-    <font>
-      <i/>
       <sz val="9"/>
       <name val="MS P Mincho"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -513,21 +473,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEEEEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD6EAF8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFDE8D8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF9E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -655,7 +600,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -717,36 +662,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -756,8 +680,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1098,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="8" style="1" customWidth="1"/>
@@ -1106,9 +1033,10 @@
     <col min="4" max="7" width="15" style="1" customWidth="1"/>
     <col min="8" max="8" width="10" style="1" customWidth="1"/>
     <col min="9" max="9" width="15" style="1" customWidth="1"/>
+    <col min="10" max="10" width="32" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1120,6 +1048,7 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -1213,7 +1142,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>17</v>
       </c>
@@ -1229,913 +1158,617 @@
       </c>
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="20"/>
-    </row>
-    <row r="9" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" s="19"/>
+      <c r="J8" s="20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F9" s="24"/>
       <c r="G9" s="24"/>
       <c r="H9" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I9" s="25"/>
-    </row>
-    <row r="10" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F10" s="24"/>
       <c r="G10" s="24"/>
       <c r="H10" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I10" s="25"/>
-    </row>
-    <row r="11" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="22" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F11" s="24"/>
       <c r="G11" s="24"/>
       <c r="H11" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I11" s="25"/>
-    </row>
-    <row r="12" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F12" s="24"/>
       <c r="G12" s="24"/>
       <c r="H12" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I12" s="25"/>
-    </row>
-    <row r="13" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F13" s="24"/>
       <c r="G13" s="24"/>
       <c r="H13" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I13" s="25"/>
-    </row>
-    <row r="14" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="21"/>
-      <c r="C14" s="26" t="s">
-        <v>43</v>
+      <c r="C14" s="27" t="s">
+        <v>44</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="25" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I14" s="25"/>
-    </row>
-    <row r="15" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" ht="84" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" s="21"/>
-      <c r="C15" s="26" t="s">
-        <v>48</v>
+      <c r="C15" s="27" t="s">
+        <v>49</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="24"/>
       <c r="H15" s="25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I15" s="25"/>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="29"/>
-      <c r="E16" s="30" t="s">
+      <c r="J15" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="32" t="s">
+    </row>
+    <row r="16" ht="84" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="D17" s="33"/>
-      <c r="E17" s="34" t="s">
+      <c r="B16" s="21"/>
+      <c r="C16" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="36" t="s">
+      <c r="D16" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38" t="s">
+      <c r="E16" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="38"/>
-    </row>
-    <row r="19" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="I16" s="25"/>
+      <c r="J16" s="26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="I17" s="25"/>
+      <c r="J17" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" ht="84" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="21"/>
+      <c r="C18" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="25"/>
+      <c r="J18" s="26" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B19" s="21"/>
-      <c r="C19" s="26" t="s">
-        <v>59</v>
+      <c r="C19" s="27" t="s">
+        <v>69</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="F19" s="24"/>
       <c r="G19" s="24"/>
       <c r="H19" s="25" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="I19" s="25"/>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="29"/>
-      <c r="E20" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="31"/>
-      <c r="C21" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="33"/>
-      <c r="E21" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38" t="s">
+      <c r="J19" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" ht="84" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="21"/>
+      <c r="C20" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="38"/>
-    </row>
-    <row r="23" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E20" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="I20" s="25"/>
+      <c r="J20" s="26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="21"/>
+      <c r="C21" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="25"/>
+      <c r="J21" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="21"/>
+      <c r="C22" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="25"/>
+      <c r="J22" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" ht="84" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="B23" s="21"/>
-      <c r="C23" s="26" t="s">
-        <v>67</v>
+      <c r="C23" s="27" t="s">
+        <v>84</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="F23" s="24"/>
       <c r="G23" s="24"/>
       <c r="H23" s="25" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="I23" s="25"/>
-    </row>
-    <row r="24" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" s="26" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="B24" s="21"/>
-      <c r="C24" s="26" t="s">
-        <v>70</v>
+      <c r="C24" s="27" t="s">
+        <v>90</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="F24" s="24"/>
       <c r="G24" s="24"/>
       <c r="H24" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I24" s="25"/>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="27"/>
-      <c r="C25" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-    </row>
-    <row r="26" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D26" s="33"/>
-      <c r="E26" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="38"/>
-    </row>
-    <row r="28" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="21"/>
+      <c r="C25" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25" s="25"/>
+      <c r="J25" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="25"/>
+      <c r="J26" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" ht="84" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" s="21"/>
+      <c r="C27" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I27" s="25"/>
+      <c r="J27" s="26" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="28" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="B28" s="21"/>
-      <c r="C28" s="26" t="s">
-        <v>77</v>
+      <c r="C28" s="27" t="s">
+        <v>104</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
       <c r="H28" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I28" s="25"/>
-    </row>
-    <row r="29" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" ht="56" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="B29" s="21"/>
-      <c r="C29" s="26" t="s">
-        <v>80</v>
+      <c r="C29" s="27" t="s">
+        <v>106</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="24"/>
       <c r="H29" s="25" t="s">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="I29" s="25"/>
-    </row>
-    <row r="30" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30" s="27"/>
-      <c r="C30" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D30" s="29"/>
-      <c r="E30" s="30" t="s">
-        <v>83</v>
-      </c>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-    </row>
-    <row r="31" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="31"/>
-      <c r="C31" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D31" s="33"/>
-      <c r="E31" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="D32" s="37"/>
-      <c r="E32" s="38" t="s">
-        <v>85</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="38"/>
-    </row>
-    <row r="33" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33" s="21"/>
-      <c r="C33" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E33" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I33" s="25"/>
-    </row>
-    <row r="34" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B34" s="21"/>
-      <c r="C34" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I34" s="25"/>
-    </row>
-    <row r="35" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="B35" s="21"/>
-      <c r="C35" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="D35" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="E35" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="I35" s="25"/>
-    </row>
-    <row r="36" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B36" s="27"/>
-      <c r="C36" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D36" s="29"/>
-      <c r="E36" s="30" t="s">
-        <v>98</v>
-      </c>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-    </row>
-    <row r="37" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B37" s="31"/>
-      <c r="C37" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D37" s="33"/>
-      <c r="E37" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="F37" s="34"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="34"/>
-      <c r="I37" s="34"/>
-    </row>
-    <row r="38" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B38" s="35"/>
-      <c r="C38" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="D38" s="37"/>
-      <c r="E38" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="F38" s="38"/>
-      <c r="G38" s="38"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="38"/>
-    </row>
-    <row r="39" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="E39" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="F39" s="24"/>
-      <c r="G39" s="24"/>
-      <c r="H39" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I39" s="25"/>
-    </row>
-    <row r="40" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="B40" s="21"/>
-      <c r="C40" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="E40" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="F40" s="24"/>
-      <c r="G40" s="24"/>
-      <c r="H40" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I40" s="25"/>
-    </row>
-    <row r="41" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="B41" s="21"/>
-      <c r="C41" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="D41" s="23" t="s">
+      <c r="J29" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="E41" s="24" t="s">
+    </row>
+    <row r="30" ht="56" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="F41" s="24"/>
-      <c r="G41" s="24"/>
-      <c r="H41" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I41" s="25"/>
-    </row>
-    <row r="42" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="21" t="s">
+      <c r="B30" s="21"/>
+      <c r="C30" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="B42" s="21"/>
-      <c r="C42" s="26" t="s">
+      <c r="D30" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="E42" s="24" t="s">
+      <c r="E30" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="F42" s="24"/>
-      <c r="G42" s="24"/>
-      <c r="H42" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I42" s="25"/>
-    </row>
-    <row r="43" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B43" s="27"/>
-      <c r="C43" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D43" s="29"/>
-      <c r="E43" s="30" t="s">
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I30" s="25"/>
+      <c r="J30" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
-      <c r="I43" s="30"/>
-    </row>
-    <row r="44" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B44" s="31"/>
-      <c r="C44" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D44" s="33"/>
-      <c r="E44" s="34" t="s">
+    </row>
+    <row r="31" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="34"/>
-    </row>
-    <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B45" s="35"/>
-      <c r="C45" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38" t="s">
+      <c r="B31" s="21"/>
+      <c r="C31" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="F45" s="38"/>
-      <c r="G45" s="38"/>
-      <c r="H45" s="38"/>
-      <c r="I45" s="38"/>
-    </row>
-    <row r="46" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
+      <c r="D31" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="B46" s="21"/>
-      <c r="C46" s="26" t="s">
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" s="25"/>
+      <c r="J31" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="D46" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="E46" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24"/>
-      <c r="H46" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I46" s="25"/>
-    </row>
-    <row r="47" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="21" t="s">
+      <c r="B32" s="21"/>
+      <c r="C32" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="B47" s="21"/>
-      <c r="C47" s="26" t="s">
+      <c r="D32" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="D47" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E47" s="24" t="s">
+      <c r="E32" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="F47" s="24"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="25" t="s">
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="I47" s="25"/>
-    </row>
-    <row r="48" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B48" s="31"/>
-      <c r="C48" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D48" s="33"/>
-      <c r="E48" s="34" t="s">
+      <c r="I32" s="25"/>
+      <c r="J32" s="26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="28" t="s">
         <v>123</v>
       </c>
-      <c r="F48" s="34"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="34"/>
-      <c r="I48" s="34"/>
-    </row>
-    <row r="49" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="B49" s="35"/>
-      <c r="C49" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="D49" s="37"/>
-      <c r="E49" s="38" t="s">
+      <c r="B33" s="28"/>
+      <c r="C33" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="F49" s="38"/>
-      <c r="G49" s="38"/>
-      <c r="H49" s="38"/>
-      <c r="I49" s="38"/>
-    </row>
-    <row r="50" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="21" t="s">
+      <c r="D33" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="30" t="s">
         <v>125</v>
       </c>
-      <c r="B50" s="21"/>
-      <c r="C50" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="E50" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="F50" s="24"/>
-      <c r="G50" s="24"/>
-      <c r="H50" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I50" s="25"/>
-    </row>
-    <row r="51" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B51" s="27"/>
-      <c r="C51" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D51" s="29"/>
-      <c r="E51" s="30" t="s">
-        <v>129</v>
-      </c>
-      <c r="F51" s="30"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="30"/>
-      <c r="I51" s="30"/>
-    </row>
-    <row r="52" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B52" s="31"/>
-      <c r="C52" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D52" s="33"/>
-      <c r="E52" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="F52" s="34"/>
-      <c r="G52" s="34"/>
-      <c r="H52" s="34"/>
-      <c r="I52" s="34"/>
-    </row>
-    <row r="53" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B53" s="21"/>
-      <c r="C53" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="D53" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="E53" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="F53" s="24"/>
-      <c r="G53" s="24"/>
-      <c r="H53" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I53" s="25"/>
-    </row>
-    <row r="54" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="B54" s="21"/>
-      <c r="C54" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="D54" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="E54" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="F54" s="24"/>
-      <c r="G54" s="24"/>
-      <c r="H54" s="25" t="s">
-        <v>138</v>
-      </c>
-      <c r="I54" s="25"/>
-    </row>
-    <row r="55" ht="35" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="39" t="s">
-        <v>139</v>
-      </c>
-      <c r="B55" s="39"/>
-      <c r="C55" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="D55" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E55" s="41" t="s">
-        <v>141</v>
-      </c>
-      <c r="F55" s="41"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="I55" s="42"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="31"/>
+      <c r="J33" s="32" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="134">
-    <mergeCell ref="A1:I1"/>
+  <mergeCells count="90">
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:D4"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="F3:G3"/>
@@ -2172,20 +1805,26 @@
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="E16:I16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:I16"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:I17"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:I20"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:I21"/>
     <mergeCell ref="A22:B22"/>
-    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:I22"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:I23"/>
@@ -2193,11 +1832,14 @@
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="A25:B25"/>
-    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="H25:I25"/>
     <mergeCell ref="A26:B26"/>
-    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:I26"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:I27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="E28:G28"/>
     <mergeCell ref="H28:I28"/>
@@ -2205,70 +1847,17 @@
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="A30:B30"/>
-    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:I30"/>
     <mergeCell ref="A31:B31"/>
-    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="H31:I31"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="H32:I32"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="E33:G33"/>
     <mergeCell ref="H33:I33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="E35:G35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="E36:I36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="E37:I37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="E38:I38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="E43:I43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="E44:I44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="E45:I45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="E48:I48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="E49:I49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="E51:I51"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="E52:I52"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="E54:G54"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="E55:G55"/>
-    <mergeCell ref="H55:I55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>